<commit_message>
datos: actualización automática 2026-09-29
</commit_message>
<xml_diff>
--- a/idecba/pgb_var.xlsx
+++ b/idecba/pgb_var.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.32.3.50\Centro_Doc\BANCO DE DATOS\CARPETAS BCO DE DATOS\PRODUCTO GEOGRÁFICO BRUTO - PGB\PGB BASE 2004\PGB trimestral\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\SRV03\Centro_Doc\BANCO DE DATOS\CARPETAS BCO DE DATOS\PRODUCTO GEOGRÁFICO BRUTO - PGB\PGB BASE 2004\PGB trimestral\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAD49A54-5DCA-41DB-BA25-85A63FE0ADA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="696" yWindow="1080" windowWidth="14904" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21150" windowHeight="2835"/>
   </bookViews>
   <sheets>
     <sheet name="PGB_K_variación_porcentual" sheetId="3" r:id="rId1"/>
@@ -54,12 +53,12 @@
     <definedName name="nuevo">#REF!</definedName>
     <definedName name="Transporte">[1]IVF!$A$22</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="56">
   <si>
     <t>Categoría</t>
   </si>
@@ -230,19 +229,19 @@
     <t>2026**</t>
   </si>
   <si>
-    <t xml:space="preserve">Variación porcentual respecto a igual trimestre del año anterior del Producto Geográfico Bruto Trimestral a precios básicos (a precios de 2004) por categoría de la ClaNAE. Ciudad de Buenos Aires.  1er. Trimestre de 2024/1er. Trimestre de 2026. </t>
-  </si>
-  <si>
     <t>Producto Geográfico Bruto - PGB</t>
   </si>
   <si>
     <t>PGB_K_variación_porcentual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variación porcentual respecto a igual trimestre del año anterior del Producto Geográfico Bruto Trimestral a precios básicos (a precios de 2004) por categoría de la ClaNAE. Ciudad de Buenos Aires.  1er. Trimestre de 2024/2do. Trimestre de 2026. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="13">
     <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="0.0"/>
@@ -629,7 +628,7 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -729,21 +728,21 @@
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="11" xfId="32" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="176" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="32" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -755,41 +754,41 @@
     </xf>
   </cellXfs>
   <cellStyles count="35">
-    <cellStyle name="Cabezal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="coltit" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="Columna títulos" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Comma" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Comma0" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="cuadro" xfId="6" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="Currency" xfId="7" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Currency0" xfId="8" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Date" xfId="9" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="datos" xfId="10" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="Encabezado" xfId="11" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="Estilo 1" xfId="12" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="Euro" xfId="13" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="F2" xfId="14" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
-    <cellStyle name="F3" xfId="15" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
-    <cellStyle name="F4" xfId="16" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="F5" xfId="17" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
-    <cellStyle name="F6" xfId="18" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
-    <cellStyle name="F7" xfId="19" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="F8" xfId="20" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
-    <cellStyle name="Fin del cuadro" xfId="21" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
-    <cellStyle name="fincuadro" xfId="22" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
-    <cellStyle name="Fixed" xfId="23" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
-    <cellStyle name="fuente" xfId="24" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
-    <cellStyle name="Heading 1" xfId="25" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
-    <cellStyle name="Heading 2" xfId="26" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="Cabezal" xfId="1"/>
+    <cellStyle name="coltit" xfId="2"/>
+    <cellStyle name="Columna títulos" xfId="3"/>
+    <cellStyle name="Comma" xfId="4"/>
+    <cellStyle name="Comma0" xfId="5"/>
+    <cellStyle name="cuadro" xfId="6"/>
+    <cellStyle name="Currency" xfId="7"/>
+    <cellStyle name="Currency0" xfId="8"/>
+    <cellStyle name="Date" xfId="9"/>
+    <cellStyle name="datos" xfId="10"/>
+    <cellStyle name="Encabezado" xfId="11"/>
+    <cellStyle name="Estilo 1" xfId="12"/>
+    <cellStyle name="Euro" xfId="13"/>
+    <cellStyle name="F2" xfId="14"/>
+    <cellStyle name="F3" xfId="15"/>
+    <cellStyle name="F4" xfId="16"/>
+    <cellStyle name="F5" xfId="17"/>
+    <cellStyle name="F6" xfId="18"/>
+    <cellStyle name="F7" xfId="19"/>
+    <cellStyle name="F8" xfId="20"/>
+    <cellStyle name="Fin del cuadro" xfId="21"/>
+    <cellStyle name="fincuadro" xfId="22"/>
+    <cellStyle name="Fixed" xfId="23"/>
+    <cellStyle name="fuente" xfId="24"/>
+    <cellStyle name="Heading 1" xfId="25"/>
+    <cellStyle name="Heading 2" xfId="26"/>
     <cellStyle name="Millares" xfId="32" builtinId="3"/>
-    <cellStyle name="Millares 27" xfId="33" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
+    <cellStyle name="Millares 27" xfId="33"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2 2" xfId="27" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
-    <cellStyle name="Normal 3" xfId="34" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
-    <cellStyle name="Percent" xfId="28" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
-    <cellStyle name="titulo" xfId="29" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
-    <cellStyle name="total" xfId="30" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
-    <cellStyle name="totcuadro" xfId="31" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
+    <cellStyle name="Normal 2 2" xfId="27"/>
+    <cellStyle name="Normal 3" xfId="34"/>
+    <cellStyle name="Percent" xfId="28"/>
+    <cellStyle name="titulo" xfId="29"/>
+    <cellStyle name="total" xfId="30"/>
+    <cellStyle name="totcuadro" xfId="31"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -810,7 +809,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="40110ciudad"/>
@@ -965,7 +964,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Estimaciones EIA"/>
@@ -1022,9 +1021,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1062,9 +1061,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1099,7 +1098,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1134,7 +1133,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1307,66 +1306,72 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N41"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O59"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="51.5546875" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" customWidth="1"/>
-    <col min="7" max="7" width="2.6640625" customWidth="1"/>
-    <col min="8" max="8" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="4.33203125" customWidth="1"/>
-    <col min="14" max="14" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" customWidth="1"/>
+    <col min="7" max="7" width="2.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="3" customWidth="1"/>
+    <col min="14" max="14" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="44" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
+    <row r="1" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="46" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
+      <c r="N1" s="46"/>
+      <c r="O1" s="46"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
       <c r="G2" s="31"/>
-      <c r="H2" s="43" t="s">
+      <c r="H2" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-      <c r="N2" s="39" t="s">
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="40"/>
+      <c r="N2" s="45" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="42"/>
+      <c r="O2" s="45"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" s="44"/>
       <c r="B3" s="32" t="s">
         <v>36</v>
       </c>
@@ -1398,11 +1403,15 @@
       <c r="L3" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="N3" s="40" t="s">
+      <c r="M3" s="41"/>
+      <c r="N3" s="39" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O3" s="32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="30" t="s">
         <v>1</v>
       </c>
@@ -1423,25 +1432,28 @@
       </c>
       <c r="G4" s="21"/>
       <c r="H4" s="20">
-        <v>4.5130851437105823</v>
+        <v>4.5579026354378716</v>
       </c>
       <c r="I4" s="20">
-        <v>6.0339247892640557</v>
+        <v>5.9470730133054595</v>
       </c>
       <c r="J4" s="20">
-        <v>4.435207348942205</v>
+        <v>4.4088439785793687</v>
       </c>
       <c r="K4" s="20">
-        <v>2.8092690818557697</v>
+        <v>2.9173353522331302</v>
       </c>
       <c r="L4" s="20">
-        <v>4.4107393085302427</v>
+        <v>4.4226627794853979</v>
       </c>
       <c r="N4" s="20">
-        <v>0.71863458042469297</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.75665610892423629</v>
+      </c>
+      <c r="O4" s="20">
+        <v>0.34668782747220295</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -1477,10 +1489,13 @@
         <v>0.67162630924417765</v>
       </c>
       <c r="N5" s="22">
-        <v>-1.2617104865518258</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>-1.1982472045935166</v>
+      </c>
+      <c r="O5" s="22">
+        <v>2.4408182027120251</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1518,8 +1533,11 @@
       <c r="N6" s="22">
         <v>-2.3742950449520683</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O6" s="22">
+        <v>-1.7833421319179976</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1549,16 +1567,19 @@
         <v>-10.904260335575911</v>
       </c>
       <c r="K7" s="22">
-        <v>-12.234300251017716</v>
+        <v>-12.210443991053788</v>
       </c>
       <c r="L7" s="20">
-        <v>-7.1131180640425118</v>
+        <v>-7.1071586284433437</v>
       </c>
       <c r="N7" s="22">
-        <v>-6.5247420025725811</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>-6.3744550910745934</v>
+      </c>
+      <c r="O7" s="22">
+        <v>-3.4704073273001623</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
@@ -1582,22 +1603,25 @@
         <v>6.9742897234703394</v>
       </c>
       <c r="I8" s="22">
-        <v>9.939849816399704</v>
+        <v>10.550370374765382</v>
       </c>
       <c r="J8" s="22">
-        <v>0.24973482659575996</v>
+        <v>0.26405139354146456</v>
       </c>
       <c r="K8" s="22">
-        <v>1.1360336645447999</v>
+        <v>1.1789071139168161</v>
       </c>
       <c r="L8" s="20">
-        <v>4.478213117144425</v>
+        <v>4.6216853401090052</v>
       </c>
       <c r="N8" s="22">
-        <v>-1.4333964256164733</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>-1.1826314525322124</v>
+      </c>
+      <c r="O8" s="22">
+        <v>0.27513069573481541</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -1633,10 +1657,13 @@
         <v>5.0779711400453786</v>
       </c>
       <c r="N9" s="22">
-        <v>-2.4127459451216637</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+        <v>-2.4255917439022223</v>
+      </c>
+      <c r="O9" s="22">
+        <v>-2.1561289585509735</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
@@ -1672,10 +1699,13 @@
         <v>2.9163011345412215E-2</v>
       </c>
       <c r="N10" s="22">
-        <v>1.5887945848201745</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+        <v>1.7488748242709296</v>
+      </c>
+      <c r="O10" s="22">
+        <v>0.78521787657741537</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
@@ -1696,25 +1726,28 @@
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="22">
-        <v>1.579125521910818</v>
+        <v>2.1677400158730986</v>
       </c>
       <c r="I11" s="22">
-        <v>3.3034733739297106</v>
+        <v>2.6330460799189659</v>
       </c>
       <c r="J11" s="22">
-        <v>4.4444508880963296</v>
+        <v>4.4001538125479467</v>
       </c>
       <c r="K11" s="22">
-        <v>8.0154787781623327</v>
+        <v>8.1675271483799161</v>
       </c>
       <c r="L11" s="20">
-        <v>4.3295177941941487</v>
+        <v>4.314361077632145</v>
       </c>
       <c r="N11" s="22">
-        <v>3.6138588146595207</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+        <v>3.0862276427686686</v>
+      </c>
+      <c r="O11" s="22">
+        <v>0.88210157113850496</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
@@ -1738,22 +1771,25 @@
         <v>11.490208836161031</v>
       </c>
       <c r="I12" s="22">
-        <v>16.127829436747977</v>
+        <v>16.129372743302927</v>
       </c>
       <c r="J12" s="22">
-        <v>32.532308911700667</v>
+        <v>32.536874469784351</v>
       </c>
       <c r="K12" s="22">
-        <v>24.35069114896109</v>
+        <v>24.367264514696551</v>
       </c>
       <c r="L12" s="20">
-        <v>21.193397575022232</v>
+        <v>21.199182039779974</v>
       </c>
       <c r="N12" s="22">
-        <v>11.258980525778007</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+        <v>10.977281167503982</v>
+      </c>
+      <c r="O12" s="22">
+        <v>7.7250392849846472</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="23" t="s">
         <v>10</v>
       </c>
@@ -1774,25 +1810,28 @@
       </c>
       <c r="G13" s="21"/>
       <c r="H13" s="22">
-        <v>2.0389611066968349</v>
+        <v>2.0112277097068532</v>
       </c>
       <c r="I13" s="22">
-        <v>3.341007622841885</v>
+        <v>3.1520283043525721</v>
       </c>
       <c r="J13" s="22">
-        <v>2.2186232399248107</v>
+        <v>2.1000010679692149</v>
       </c>
       <c r="K13" s="22">
-        <v>0.26578444687492819</v>
+        <v>0.29850992288422695</v>
       </c>
       <c r="L13" s="20">
-        <v>1.9414812413363958</v>
+        <v>1.8673293308914429</v>
       </c>
       <c r="N13" s="22">
-        <v>-0.82446439655484705</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+        <v>-0.68540884916706846</v>
+      </c>
+      <c r="O13" s="22">
+        <v>-0.71099183079181838</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="23" t="s">
         <v>11</v>
       </c>
@@ -1828,10 +1867,13 @@
         <v>-0.40353488553199757</v>
       </c>
       <c r="N14" s="22">
-        <v>-0.16883300003485147</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.79764892133489251</v>
+      </c>
+      <c r="O14" s="22">
+        <v>-0.64187370256812981</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>12</v>
       </c>
@@ -1855,22 +1897,25 @@
         <v>1.0741567079422421</v>
       </c>
       <c r="I15" s="22">
-        <v>0.55877194323181723</v>
+        <v>0.55855970062947957</v>
       </c>
       <c r="J15" s="22">
-        <v>0.9950947732881632</v>
+        <v>0.99432711856199951</v>
       </c>
       <c r="K15" s="22">
-        <v>1.0012885992974008</v>
+        <v>1.0034269256763206</v>
       </c>
       <c r="L15" s="20">
-        <v>0.91118288834006744</v>
+        <v>0.91148919867156675</v>
       </c>
       <c r="N15" s="22">
-        <v>0.8627094578360861</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.87241160868056777</v>
+      </c>
+      <c r="O15" s="22">
+        <v>0.58511841991952807</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>13</v>
       </c>
@@ -1894,22 +1939,25 @@
         <v>-0.40270962090180884</v>
       </c>
       <c r="I16" s="22">
-        <v>0.48660566479474809</v>
+        <v>0.48662155892125192</v>
       </c>
       <c r="J16" s="22">
-        <v>1.9285931201852957</v>
+        <v>1.9286266478117264</v>
       </c>
       <c r="K16" s="22">
-        <v>0.51839273612208636</v>
+        <v>0.81037979661644499</v>
       </c>
       <c r="L16" s="20">
-        <v>0.60941359130168848</v>
+        <v>0.68675052521709468</v>
       </c>
       <c r="N16" s="22">
-        <v>1.1728688146387389</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+        <v>1.1650156956300783</v>
+      </c>
+      <c r="O16" s="22">
+        <v>0.99146138322123711</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>14</v>
       </c>
@@ -1933,22 +1981,25 @@
         <v>-7.9884986694345184E-2</v>
       </c>
       <c r="I17" s="22">
-        <v>2.6752661675452094</v>
+        <v>2.6816472874868769</v>
       </c>
       <c r="J17" s="22">
-        <v>-2.5072222491490215</v>
+        <v>-2.4935237597385917</v>
       </c>
       <c r="K17" s="22">
-        <v>-1.8696190970729831</v>
+        <v>-1.8584006255346397</v>
       </c>
       <c r="L17" s="20">
-        <v>-0.42490720032563045</v>
+        <v>-0.4171876596941515</v>
       </c>
       <c r="N17" s="22">
-        <v>-4.0534289678970659</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+        <v>-3.6726256140452662</v>
+      </c>
+      <c r="O17" s="22">
+        <v>-3.2706521846812331</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="34" t="s">
         <v>15</v>
       </c>
@@ -1972,22 +2023,26 @@
         <v>1.4347179366301699</v>
       </c>
       <c r="I18" s="35">
-        <v>1.977264485968111</v>
+        <v>1.9795738010533581</v>
       </c>
       <c r="J18" s="35">
-        <v>0.61567635601569304</v>
+        <v>0.63019773478174557</v>
       </c>
       <c r="K18" s="35">
-        <v>-10.245767326027877</v>
+        <v>-2.6571908249348297</v>
       </c>
       <c r="L18" s="36">
-        <v>-1.5339672070753374</v>
-      </c>
+        <v>0.37440164403468312</v>
+      </c>
+      <c r="M18" s="41"/>
       <c r="N18" s="35">
-        <v>-1.6917237687808062</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+        <v>-1.5239266775241789</v>
+      </c>
+      <c r="O18" s="35">
+        <v>-2.1369178954242285</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>49</v>
       </c>
@@ -2001,7 +2056,7 @@
       <c r="I19" s="22"/>
       <c r="J19" s="22"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>50</v>
       </c>
@@ -2012,7 +2067,7 @@
       <c r="F20" s="25"/>
       <c r="G20" s="25"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="13" t="s">
         <v>44</v>
       </c>
@@ -2025,157 +2080,247 @@
       <c r="H21" s="19"/>
       <c r="I21" s="19"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="26"/>
-      <c r="I24" s="26"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="26"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B26" s="26"/>
-      <c r="C26" s="26"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="26"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B27" s="26"/>
-      <c r="C27" s="26"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="26"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="26"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="26"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="26"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B31" s="26"/>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="26"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="26"/>
-    </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-    </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B34" s="26"/>
-      <c r="C34" s="26"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="26"/>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B35" s="26"/>
-      <c r="C35" s="26"/>
-      <c r="D35" s="26"/>
-      <c r="E35" s="26"/>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="26"/>
-      <c r="I35" s="26"/>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B36" s="26"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="26"/>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B37" s="26"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="26"/>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B38" s="26"/>
-      <c r="C38" s="26"/>
-      <c r="D38" s="26"/>
-      <c r="E38" s="26"/>
-      <c r="F38" s="26"/>
-      <c r="G38" s="26"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="26"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B24" s="42"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="42"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="42"/>
+      <c r="H24" s="42"/>
+      <c r="I24" s="42"/>
+      <c r="J24" s="42"/>
+      <c r="K24" s="42"/>
+      <c r="L24" s="42"/>
+      <c r="M24" s="42"/>
+      <c r="N24" s="42"/>
+      <c r="O24" s="42"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B25" s="42"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="42"/>
+      <c r="I25" s="42"/>
+      <c r="J25" s="42"/>
+      <c r="K25" s="42"/>
+      <c r="L25" s="42"/>
+      <c r="M25" s="42"/>
+      <c r="N25" s="42"/>
+      <c r="O25" s="42"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B26" s="42"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="42"/>
+      <c r="F26" s="42"/>
+      <c r="G26" s="42"/>
+      <c r="H26" s="42"/>
+      <c r="I26" s="42"/>
+      <c r="J26" s="42"/>
+      <c r="K26" s="42"/>
+      <c r="L26" s="42"/>
+      <c r="M26" s="42"/>
+      <c r="N26" s="42"/>
+      <c r="O26" s="42"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B27" s="42"/>
+      <c r="C27" s="42"/>
+      <c r="D27" s="42"/>
+      <c r="E27" s="42"/>
+      <c r="F27" s="42"/>
+      <c r="G27" s="42"/>
+      <c r="H27" s="42"/>
+      <c r="I27" s="42"/>
+      <c r="J27" s="42"/>
+      <c r="K27" s="42"/>
+      <c r="L27" s="42"/>
+      <c r="M27" s="42"/>
+      <c r="N27" s="42"/>
+      <c r="O27" s="42"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B28" s="42"/>
+      <c r="C28" s="42"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="42"/>
+      <c r="G28" s="42"/>
+      <c r="H28" s="42"/>
+      <c r="I28" s="42"/>
+      <c r="J28" s="42"/>
+      <c r="K28" s="42"/>
+      <c r="L28" s="42"/>
+      <c r="M28" s="42"/>
+      <c r="N28" s="42"/>
+      <c r="O28" s="42"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B29" s="42"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="42"/>
+      <c r="F29" s="42"/>
+      <c r="G29" s="42"/>
+      <c r="H29" s="42"/>
+      <c r="I29" s="42"/>
+      <c r="J29" s="42"/>
+      <c r="K29" s="42"/>
+      <c r="L29" s="42"/>
+      <c r="M29" s="42"/>
+      <c r="N29" s="42"/>
+      <c r="O29" s="42"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B30" s="42"/>
+      <c r="C30" s="42"/>
+      <c r="D30" s="42"/>
+      <c r="E30" s="42"/>
+      <c r="F30" s="42"/>
+      <c r="G30" s="42"/>
+      <c r="H30" s="42"/>
+      <c r="I30" s="42"/>
+      <c r="J30" s="42"/>
+      <c r="K30" s="42"/>
+      <c r="L30" s="42"/>
+      <c r="M30" s="42"/>
+      <c r="N30" s="42"/>
+      <c r="O30" s="42"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B31" s="42"/>
+      <c r="C31" s="42"/>
+      <c r="D31" s="42"/>
+      <c r="E31" s="42"/>
+      <c r="F31" s="42"/>
+      <c r="G31" s="42"/>
+      <c r="H31" s="42"/>
+      <c r="I31" s="42"/>
+      <c r="J31" s="42"/>
+      <c r="K31" s="42"/>
+      <c r="L31" s="42"/>
+      <c r="M31" s="42"/>
+      <c r="N31" s="42"/>
+      <c r="O31" s="42"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B32" s="42"/>
+      <c r="C32" s="42"/>
+      <c r="D32" s="42"/>
+      <c r="E32" s="42"/>
+      <c r="F32" s="42"/>
+      <c r="G32" s="42"/>
+      <c r="H32" s="42"/>
+      <c r="I32" s="42"/>
+      <c r="J32" s="42"/>
+      <c r="K32" s="42"/>
+      <c r="L32" s="42"/>
+      <c r="M32" s="42"/>
+      <c r="N32" s="42"/>
+      <c r="O32" s="42"/>
+    </row>
+    <row r="33" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B33" s="42"/>
+      <c r="C33" s="42"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="42"/>
+      <c r="F33" s="42"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="42"/>
+      <c r="L33" s="42"/>
+      <c r="M33" s="42"/>
+      <c r="N33" s="42"/>
+      <c r="O33" s="42"/>
+    </row>
+    <row r="34" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B34" s="42"/>
+      <c r="C34" s="42"/>
+      <c r="D34" s="42"/>
+      <c r="E34" s="42"/>
+      <c r="F34" s="42"/>
+      <c r="G34" s="42"/>
+      <c r="H34" s="42"/>
+      <c r="I34" s="42"/>
+      <c r="J34" s="42"/>
+      <c r="K34" s="42"/>
+      <c r="L34" s="42"/>
+      <c r="M34" s="42"/>
+      <c r="N34" s="42"/>
+      <c r="O34" s="42"/>
+    </row>
+    <row r="35" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B35" s="42"/>
+      <c r="C35" s="42"/>
+      <c r="D35" s="42"/>
+      <c r="E35" s="42"/>
+      <c r="F35" s="42"/>
+      <c r="G35" s="42"/>
+      <c r="H35" s="42"/>
+      <c r="I35" s="42"/>
+      <c r="J35" s="42"/>
+      <c r="K35" s="42"/>
+      <c r="L35" s="42"/>
+      <c r="M35" s="42"/>
+      <c r="N35" s="42"/>
+      <c r="O35" s="42"/>
+    </row>
+    <row r="36" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B36" s="42"/>
+      <c r="C36" s="42"/>
+      <c r="D36" s="42"/>
+      <c r="E36" s="42"/>
+      <c r="F36" s="42"/>
+      <c r="G36" s="42"/>
+      <c r="H36" s="42"/>
+      <c r="I36" s="42"/>
+      <c r="J36" s="42"/>
+      <c r="K36" s="42"/>
+      <c r="L36" s="42"/>
+      <c r="M36" s="42"/>
+      <c r="N36" s="42"/>
+      <c r="O36" s="42"/>
+    </row>
+    <row r="37" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B37" s="42"/>
+      <c r="C37" s="42"/>
+      <c r="D37" s="42"/>
+      <c r="E37" s="42"/>
+      <c r="F37" s="42"/>
+      <c r="G37" s="42"/>
+      <c r="H37" s="42"/>
+      <c r="I37" s="42"/>
+      <c r="J37" s="42"/>
+      <c r="K37" s="42"/>
+      <c r="L37" s="42"/>
+      <c r="M37" s="42"/>
+      <c r="N37" s="42"/>
+      <c r="O37" s="42"/>
+    </row>
+    <row r="38" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B38" s="42"/>
+      <c r="C38" s="42"/>
+      <c r="D38" s="42"/>
+      <c r="E38" s="42"/>
+      <c r="F38" s="42"/>
+      <c r="G38" s="42"/>
+      <c r="H38" s="42"/>
+      <c r="I38" s="42"/>
+      <c r="J38" s="42"/>
+      <c r="K38" s="42"/>
+      <c r="L38" s="42"/>
+      <c r="M38" s="42"/>
+      <c r="N38" s="42"/>
+      <c r="O38" s="42"/>
+    </row>
+    <row r="39" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B39" s="26"/>
       <c r="C39" s="26"/>
       <c r="D39" s="26"/>
@@ -2185,11 +2330,8 @@
       <c r="H39" s="26"/>
       <c r="I39" s="26"/>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B40" s="38">
-        <f>+B23-B4</f>
-        <v>6.3531678994888647</v>
-      </c>
+    <row r="40" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B40" s="38"/>
       <c r="C40" s="26"/>
       <c r="D40" s="26"/>
       <c r="E40" s="26"/>
@@ -2198,22 +2340,317 @@
       <c r="H40" s="26"/>
       <c r="I40" s="26"/>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="26"/>
-      <c r="C41" s="26"/>
-      <c r="D41" s="26"/>
-      <c r="E41" s="26"/>
-      <c r="F41" s="26"/>
-      <c r="G41" s="26"/>
-      <c r="H41" s="26"/>
-      <c r="I41" s="26"/>
+    <row r="41" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B41" s="42"/>
+      <c r="C41" s="42"/>
+      <c r="D41" s="42"/>
+      <c r="E41" s="42"/>
+      <c r="F41" s="42"/>
+      <c r="G41" s="42"/>
+      <c r="H41" s="42"/>
+      <c r="I41" s="42"/>
+      <c r="J41" s="42"/>
+      <c r="K41" s="42"/>
+      <c r="L41" s="42"/>
+      <c r="M41" s="42"/>
+      <c r="N41" s="42"/>
+      <c r="O41" s="42"/>
+    </row>
+    <row r="42" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B42" s="42"/>
+      <c r="C42" s="42"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="42"/>
+      <c r="F42" s="42"/>
+      <c r="G42" s="42"/>
+      <c r="H42" s="42"/>
+      <c r="I42" s="42"/>
+      <c r="J42" s="42"/>
+      <c r="K42" s="42"/>
+      <c r="L42" s="42"/>
+      <c r="M42" s="42"/>
+      <c r="N42" s="42"/>
+      <c r="O42" s="42"/>
+    </row>
+    <row r="43" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B43" s="42"/>
+      <c r="C43" s="42"/>
+      <c r="D43" s="42"/>
+      <c r="E43" s="42"/>
+      <c r="F43" s="42"/>
+      <c r="G43" s="42"/>
+      <c r="H43" s="42"/>
+      <c r="I43" s="42"/>
+      <c r="J43" s="42"/>
+      <c r="K43" s="42"/>
+      <c r="L43" s="42"/>
+      <c r="M43" s="42"/>
+      <c r="N43" s="42"/>
+      <c r="O43" s="42"/>
+    </row>
+    <row r="44" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B44" s="42"/>
+      <c r="C44" s="42"/>
+      <c r="D44" s="42"/>
+      <c r="E44" s="42"/>
+      <c r="F44" s="42"/>
+      <c r="G44" s="42"/>
+      <c r="H44" s="42"/>
+      <c r="I44" s="42"/>
+      <c r="J44" s="42"/>
+      <c r="K44" s="42"/>
+      <c r="L44" s="42"/>
+      <c r="M44" s="42"/>
+      <c r="N44" s="42"/>
+      <c r="O44" s="42"/>
+    </row>
+    <row r="45" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B45" s="42"/>
+      <c r="C45" s="42"/>
+      <c r="D45" s="42"/>
+      <c r="E45" s="42"/>
+      <c r="F45" s="42"/>
+      <c r="G45" s="42"/>
+      <c r="H45" s="42"/>
+      <c r="I45" s="42"/>
+      <c r="J45" s="42"/>
+      <c r="K45" s="42"/>
+      <c r="L45" s="42"/>
+      <c r="M45" s="42"/>
+      <c r="N45" s="42"/>
+      <c r="O45" s="42"/>
+    </row>
+    <row r="46" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B46" s="42"/>
+      <c r="C46" s="42"/>
+      <c r="D46" s="42"/>
+      <c r="E46" s="42"/>
+      <c r="F46" s="42"/>
+      <c r="G46" s="42"/>
+      <c r="H46" s="42"/>
+      <c r="I46" s="42"/>
+      <c r="J46" s="42"/>
+      <c r="K46" s="42"/>
+      <c r="L46" s="42"/>
+      <c r="M46" s="42"/>
+      <c r="N46" s="42"/>
+      <c r="O46" s="42"/>
+    </row>
+    <row r="47" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B47" s="42"/>
+      <c r="C47" s="42"/>
+      <c r="D47" s="42"/>
+      <c r="E47" s="42"/>
+      <c r="F47" s="42"/>
+      <c r="G47" s="42"/>
+      <c r="H47" s="42"/>
+      <c r="I47" s="42"/>
+      <c r="J47" s="42"/>
+      <c r="K47" s="42"/>
+      <c r="L47" s="42"/>
+      <c r="M47" s="42"/>
+      <c r="N47" s="42"/>
+      <c r="O47" s="42"/>
+    </row>
+    <row r="48" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B48" s="42"/>
+      <c r="C48" s="42"/>
+      <c r="D48" s="42"/>
+      <c r="E48" s="42"/>
+      <c r="F48" s="42"/>
+      <c r="G48" s="42"/>
+      <c r="H48" s="42"/>
+      <c r="I48" s="42"/>
+      <c r="J48" s="42"/>
+      <c r="K48" s="42"/>
+      <c r="L48" s="42"/>
+      <c r="M48" s="42"/>
+      <c r="N48" s="42"/>
+      <c r="O48" s="42"/>
+    </row>
+    <row r="49" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B49" s="42"/>
+      <c r="C49" s="42"/>
+      <c r="D49" s="42"/>
+      <c r="E49" s="42"/>
+      <c r="F49" s="42"/>
+      <c r="G49" s="42"/>
+      <c r="H49" s="42"/>
+      <c r="I49" s="42"/>
+      <c r="J49" s="42"/>
+      <c r="K49" s="42"/>
+      <c r="L49" s="42"/>
+      <c r="M49" s="42"/>
+      <c r="N49" s="42"/>
+      <c r="O49" s="42"/>
+    </row>
+    <row r="50" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B50" s="42"/>
+      <c r="C50" s="42"/>
+      <c r="D50" s="42"/>
+      <c r="E50" s="42"/>
+      <c r="F50" s="42"/>
+      <c r="G50" s="42"/>
+      <c r="H50" s="42"/>
+      <c r="I50" s="42"/>
+      <c r="J50" s="42"/>
+      <c r="K50" s="42"/>
+      <c r="L50" s="42"/>
+      <c r="M50" s="42"/>
+      <c r="N50" s="42"/>
+      <c r="O50" s="42"/>
+    </row>
+    <row r="51" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B51" s="42"/>
+      <c r="C51" s="42"/>
+      <c r="D51" s="42"/>
+      <c r="E51" s="42"/>
+      <c r="F51" s="42"/>
+      <c r="G51" s="42"/>
+      <c r="H51" s="42"/>
+      <c r="I51" s="42"/>
+      <c r="J51" s="42"/>
+      <c r="K51" s="42"/>
+      <c r="L51" s="42"/>
+      <c r="M51" s="42"/>
+      <c r="N51" s="42"/>
+      <c r="O51" s="42"/>
+    </row>
+    <row r="52" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B52" s="42"/>
+      <c r="C52" s="42"/>
+      <c r="D52" s="42"/>
+      <c r="E52" s="42"/>
+      <c r="F52" s="42"/>
+      <c r="G52" s="42"/>
+      <c r="H52" s="42"/>
+      <c r="I52" s="42"/>
+      <c r="J52" s="42"/>
+      <c r="K52" s="42"/>
+      <c r="L52" s="42"/>
+      <c r="M52" s="42"/>
+      <c r="N52" s="42"/>
+      <c r="O52" s="42"/>
+    </row>
+    <row r="53" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B53" s="42"/>
+      <c r="C53" s="42"/>
+      <c r="D53" s="42"/>
+      <c r="E53" s="42"/>
+      <c r="F53" s="42"/>
+      <c r="G53" s="42"/>
+      <c r="H53" s="42"/>
+      <c r="I53" s="42"/>
+      <c r="J53" s="42"/>
+      <c r="K53" s="42"/>
+      <c r="L53" s="42"/>
+      <c r="M53" s="42"/>
+      <c r="N53" s="42"/>
+      <c r="O53" s="42"/>
+    </row>
+    <row r="54" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B54" s="42"/>
+      <c r="C54" s="42"/>
+      <c r="D54" s="42"/>
+      <c r="E54" s="42"/>
+      <c r="F54" s="42"/>
+      <c r="G54" s="42"/>
+      <c r="H54" s="42"/>
+      <c r="I54" s="42"/>
+      <c r="J54" s="42"/>
+      <c r="K54" s="42"/>
+      <c r="L54" s="42"/>
+      <c r="M54" s="42"/>
+      <c r="N54" s="42"/>
+      <c r="O54" s="42"/>
+    </row>
+    <row r="55" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B55" s="42"/>
+      <c r="C55" s="42"/>
+      <c r="D55" s="42"/>
+      <c r="E55" s="42"/>
+      <c r="F55" s="42"/>
+      <c r="G55" s="42"/>
+      <c r="H55" s="42"/>
+      <c r="I55" s="42"/>
+      <c r="J55" s="42"/>
+      <c r="K55" s="42"/>
+      <c r="L55" s="42"/>
+      <c r="M55" s="42"/>
+      <c r="N55" s="42"/>
+      <c r="O55" s="42"/>
+    </row>
+    <row r="56" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B56" s="42"/>
+      <c r="C56" s="42"/>
+      <c r="D56" s="42"/>
+      <c r="E56" s="42"/>
+      <c r="F56" s="42"/>
+      <c r="G56" s="42"/>
+      <c r="H56" s="42"/>
+      <c r="I56" s="42"/>
+      <c r="J56" s="42"/>
+      <c r="K56" s="42"/>
+      <c r="L56" s="42"/>
+      <c r="M56" s="42"/>
+      <c r="N56" s="42"/>
+      <c r="O56" s="42"/>
+    </row>
+    <row r="57" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B57" s="42"/>
+      <c r="C57" s="42"/>
+      <c r="D57" s="42"/>
+      <c r="E57" s="42"/>
+      <c r="F57" s="42"/>
+      <c r="G57" s="42"/>
+      <c r="H57" s="42"/>
+      <c r="I57" s="42"/>
+      <c r="J57" s="42"/>
+      <c r="K57" s="42"/>
+      <c r="L57" s="42"/>
+      <c r="M57" s="42"/>
+      <c r="N57" s="42"/>
+      <c r="O57" s="42"/>
+    </row>
+    <row r="58" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B58" s="42"/>
+      <c r="C58" s="42"/>
+      <c r="D58" s="42"/>
+      <c r="E58" s="42"/>
+      <c r="F58" s="42"/>
+      <c r="G58" s="42"/>
+      <c r="H58" s="42"/>
+      <c r="I58" s="42"/>
+      <c r="J58" s="42"/>
+      <c r="K58" s="42"/>
+      <c r="L58" s="42"/>
+      <c r="M58" s="42"/>
+      <c r="N58" s="42"/>
+      <c r="O58" s="42"/>
+    </row>
+    <row r="59" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B59" s="42"/>
+      <c r="C59" s="42"/>
+      <c r="D59" s="42"/>
+      <c r="E59" s="42"/>
+      <c r="F59" s="42"/>
+      <c r="G59" s="42"/>
+      <c r="H59" s="42"/>
+      <c r="I59" s="42"/>
+      <c r="J59" s="42"/>
+      <c r="K59" s="42"/>
+      <c r="L59" s="42"/>
+      <c r="M59" s="42"/>
+      <c r="N59" s="42"/>
+      <c r="O59" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="H2:L2"/>
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2221,37 +2658,37 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="53.109375" customWidth="1"/>
-    <col min="2" max="2" width="60.109375" customWidth="1"/>
+    <col min="1" max="1" width="53.140625" customWidth="1"/>
+    <col min="2" max="2" width="60.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+    <row r="1" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="46"/>
-    </row>
-    <row r="2" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="48"/>
+    </row>
+    <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>19</v>
       </c>
@@ -2259,7 +2696,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>21</v>
       </c>
@@ -2267,7 +2704,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -2275,7 +2712,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>23</v>
       </c>
@@ -2283,7 +2720,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>33</v>
       </c>
@@ -2291,7 +2728,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="41.4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
         <v>24</v>
       </c>
@@ -2299,7 +2736,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
         <v>25</v>
       </c>
@@ -2307,7 +2744,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>26</v>
       </c>
@@ -2315,7 +2752,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="34.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>27</v>
       </c>
@@ -2323,7 +2760,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="34.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>28</v>
       </c>
@@ -2331,7 +2768,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="15" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
         <v>29</v>
       </c>
@@ -2339,7 +2776,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="49.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" ht="49.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>30</v>
       </c>
@@ -2347,10 +2784,10 @@
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B19" s="12"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="12"/>
     </row>
   </sheetData>

</xml_diff>